<commit_message>
inquiry: new message from akku
</commit_message>
<xml_diff>
--- a/Messages/messages.xlsx
+++ b/Messages/messages.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="35.83203125" customWidth="1"/>
@@ -423,9 +423,26 @@
         <v>Time</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>akku</v>
+      </c>
+      <c r="B2" t="str">
+        <v>akku@gmail.com</v>
+      </c>
+      <c r="C2" t="str">
+        <v>dwdfwgrgfgg</v>
+      </c>
+      <c r="D2" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="E2" t="str">
+        <v>10:15 pm</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
inquiry: new message from aaaa
</commit_message>
<xml_diff>
--- a/Messages/messages.xlsx
+++ b/Messages/messages.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="35.83203125" customWidth="1"/>
@@ -440,9 +440,26 @@
         <v>10:15 pm</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>aaaa</v>
+      </c>
+      <c r="B3" t="str">
+        <v>a@gmail.com</v>
+      </c>
+      <c r="C3" t="str">
+        <v>djuifh fioeflfksjfkgblf</v>
+      </c>
+      <c r="D3" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="E3" t="str">
+        <v>10:22 pm</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
inquiry: new message from Arun
</commit_message>
<xml_diff>
--- a/Messages/messages.xlsx
+++ b/Messages/messages.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="35.83203125" customWidth="1"/>
@@ -457,9 +457,26 @@
         <v>10:22 pm</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Arun</v>
+      </c>
+      <c r="B4" t="str">
+        <v>arun@gmail.com</v>
+      </c>
+      <c r="C4" t="str">
+        <v>I want your help to buld an app</v>
+      </c>
+      <c r="D4" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="E4" t="str">
+        <v>10:26 pm</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
inquiry: new message from Sjsjjsmdj
</commit_message>
<xml_diff>
--- a/Messages/messages.xlsx
+++ b/Messages/messages.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="35.83203125" customWidth="1"/>
@@ -474,9 +474,26 @@
         <v>10:26 pm</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Sjsjjsmdj</v>
+      </c>
+      <c r="B5" t="str">
+        <v>ajaja@gmail.com</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Zkdjdjdjddj</v>
+      </c>
+      <c r="D5" t="str">
+        <v>29/09/2026</v>
+      </c>
+      <c r="E5" t="str">
+        <v>01:24 am</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
inquiry: new message from kunnaoan
</commit_message>
<xml_diff>
--- a/Messages/messages.xlsx
+++ b/Messages/messages.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="35.83203125" customWidth="1"/>
@@ -491,9 +491,26 @@
         <v>01:24 am</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>kunnaoan</v>
+      </c>
+      <c r="B6" t="str">
+        <v>kuttan4727@gmail.com</v>
+      </c>
+      <c r="C6" t="str">
+        <v>gfhhfdhggfhxh</v>
+      </c>
+      <c r="D6" t="str">
+        <v>29/09/2026</v>
+      </c>
+      <c r="E6" t="str">
+        <v>10:41 am</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
inquiry: new message from Jghhh
</commit_message>
<xml_diff>
--- a/Messages/messages.xlsx
+++ b/Messages/messages.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="35.83203125" customWidth="1"/>
@@ -508,9 +508,26 @@
         <v>10:41 am</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Jghhh</v>
+      </c>
+      <c r="B7" t="str">
+        <v>arun@gmail.com</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Jfhnnbhnbbbb</v>
+      </c>
+      <c r="D7" t="str">
+        <v>29/09/2026</v>
+      </c>
+      <c r="E7" t="str">
+        <v>11:04 pm</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>